<commit_message>
Finialized the Project Page UI
I finished the Project Page Ui and implmneted date checks, and file uploads. Aslo, updated the sprint backlog and burndown.
</commit_message>
<xml_diff>
--- a/documentation/Project Sprint Backlog - Sprint 1.xlsx
+++ b/documentation/Project Sprint Backlog - Sprint 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\Dev New folder (3)\DevOps_Project_Portfolio_Hub_Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90232BF1-A305-47A4-A7BD-A625574F83B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D7CCA8-1A37-4F0C-9E0F-AFB8DA1D4E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11220" yWindow="0" windowWidth="15960" windowHeight="14010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="65145" yWindow="4035" windowWidth="21330" windowHeight="12195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
   <si>
     <t>Task Manager / Dev</t>
   </si>
@@ -77,22 +77,46 @@
     <t>Bind Page flow</t>
   </si>
   <si>
-    <t>Implment Log-Out</t>
-  </si>
-  <si>
-    <t>Implment Log-In</t>
-  </si>
-  <si>
     <t>Implment Edit Account Portfolio Page</t>
   </si>
   <si>
     <t>Implment Edit Project Page</t>
   </si>
   <si>
-    <t>Implment Create Account</t>
-  </si>
-  <si>
-    <t>Bind Edits to UI and Update Pages</t>
+    <t>Bind Edits to UI and Update  Account Portfolio Page</t>
+  </si>
+  <si>
+    <t>Bind Edits to UI and Update Project Pages</t>
+  </si>
+  <si>
+    <t>Amount Remaining After…</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Hours Worked</t>
+  </si>
+  <si>
+    <t>Initalized the project with working code</t>
+  </si>
+  <si>
+    <t>Implemented the UI for the Home Screen</t>
+  </si>
+  <si>
+    <t>Implemented the UI for the Account Portfolio</t>
+  </si>
+  <si>
+    <t>Implemented the UI for the Project Page</t>
+  </si>
+  <si>
+    <t>Binded the Pages to flow with GuiHelper</t>
+  </si>
+  <si>
+    <t>Implmented file upload for the projects</t>
+  </si>
+  <si>
+    <t>Implmented rest of the Project page View UI and Binding</t>
   </si>
 </sst>
 </file>
@@ -129,7 +153,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -166,8 +190,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -208,11 +244,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -226,11 +277,19 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.453125" customWidth="1"/>
@@ -519,28 +578,37 @@
     <col min="4" max="4" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="9" t="s">
+      <c r="C1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="14" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="10">
+      <c r="E1" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -552,9 +620,12 @@
       <c r="D3" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="10">
+      <c r="E3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -566,9 +637,10 @@
       <c r="D4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="10">
+      <c r="E4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -580,9 +652,12 @@
       <c r="D5" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="10">
+      <c r="E5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -594,9 +669,12 @@
       <c r="D6" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="10">
+      <c r="E6" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="9">
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -608,9 +686,12 @@
       <c r="D7" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="10">
+      <c r="E7" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -622,9 +703,10 @@
       <c r="D8" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="10">
+      <c r="E8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -636,23 +718,27 @@
       <c r="D9" s="5">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="10">
+      <c r="E9" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D10" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="10">
+      <c r="E10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -664,79 +750,176 @@
       <c r="D11" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="10">
+      <c r="E11" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
         <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
+        <v>1</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B14" s="6"/>
+      <c r="C14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="8">
+        <f>SUM(D3:D13)</f>
+        <v>15</v>
+      </c>
+      <c r="E14" s="8">
+        <f>SUM(E3:E13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B16" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="10">
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="5">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="10">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="10">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="10">
-        <v>1</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="10">
-        <v>1</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="6"/>
-      <c r="C16" s="7" t="s">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="10">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="10">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B25" s="1"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="8">
-        <f>SUM(D3:D15)</f>
-        <v>19.5</v>
-      </c>
+      <c r="D26" s="8">
+        <f>SUM(D18:D25)</f>
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B52" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added the UI for Login and Create Account
Created only the UI for the Login and the Create Account Pages.
</commit_message>
<xml_diff>
--- a/documentation/Project Sprint Backlog - Sprint 1.xlsx
+++ b/documentation/Project Sprint Backlog - Sprint 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\DevOps_Project\DevOps_Project_Portfolio_Hub_Project\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\temp Dev Folder\DevOps_Project_Portfolio_Hub_Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366363C2-1182-45D9-A4DF-62A7CC7E9594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E750DC4-3C9C-42EE-BDD4-3649994AE275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="65145" yWindow="4035" windowWidth="21330" windowHeight="12195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13330" yWindow="0" windowWidth="12270" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
   <si>
     <t>Task Manager / Dev</t>
   </si>
@@ -117,13 +117,16 @@
   </si>
   <si>
     <t>Implmented rest of the Project page View UI and Binding</t>
+  </si>
+  <si>
+    <t>Week 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,6 +151,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -606,6 +615,9 @@
       <c r="E2" s="11" t="s">
         <v>18</v>
       </c>
+      <c r="F2" s="11" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
@@ -623,10 +635,11 @@
       <c r="E3" s="12">
         <v>0</v>
       </c>
+      <c r="F3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
@@ -640,6 +653,7 @@
       <c r="E4" s="12">
         <v>1</v>
       </c>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
@@ -657,6 +671,7 @@
       <c r="E5" s="12">
         <v>0</v>
       </c>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
@@ -674,6 +689,7 @@
       <c r="E6" s="12">
         <v>0</v>
       </c>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
@@ -691,10 +707,11 @@
       <c r="E7" s="12">
         <v>0</v>
       </c>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>3</v>
@@ -708,6 +725,7 @@
       <c r="E8" s="12">
         <v>2</v>
       </c>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
@@ -725,10 +743,11 @@
       <c r="E9" s="12">
         <v>0</v>
       </c>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>3</v>
@@ -742,6 +761,7 @@
       <c r="E10" s="12">
         <v>1</v>
       </c>
+      <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
@@ -759,6 +779,7 @@
       <c r="E11" s="12">
         <v>0</v>
       </c>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
@@ -776,6 +797,7 @@
       <c r="E12" s="12">
         <v>1</v>
       </c>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
@@ -793,6 +815,7 @@
       <c r="E13" s="12">
         <v>0</v>
       </c>
+      <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B14" s="6"/>
@@ -806,6 +829,10 @@
       <c r="E14" s="8">
         <f>SUM(E3:E13)</f>
         <v>5</v>
+      </c>
+      <c r="F14" s="8">
+        <f>SUM(F3:F13)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -929,6 +956,7 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>